<commit_message>
docs: reemitir matriz de trazabilidad con columna ID-Flujo (45 flujos alternativos/excepciones del ERS)
</commit_message>
<xml_diff>
--- a/04_Trazabilidad/Matriz_Trazabilidad_v2.xlsx
+++ b/04_Trazabilidad/Matriz_Trazabilidad_v2.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Trazabilidad_v2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Matriz_Trazabilidad_v2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matriz_Trazabilidad_v2'!$A$1:$L$61</definedName>
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -533,6 +533,11 @@
           <t>ID-Caso-Prueba</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ID-Flujo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -600,6 +605,11 @@
           <t>CP-RF-01</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>CU-01.4e</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -667,6 +677,11 @@
           <t>CP-RF-02</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>CU-01.2e</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -734,6 +749,11 @@
           <t>CP-RF-03</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>CU-02.2e</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -801,6 +821,11 @@
           <t>CP-RF-04</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>CU-03.4e</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -868,6 +893,11 @@
           <t>CP-RF-05</t>
         </is>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>CU-04.1e</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -935,6 +965,11 @@
           <t>CP-RF-06</t>
         </is>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>CU-04.2e</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1002,6 +1037,11 @@
           <t>CP-RF-07</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>CU-05.2e</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1069,6 +1109,11 @@
           <t>CP-RF-08</t>
         </is>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>CU-05.3e</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1136,6 +1181,11 @@
           <t>CP-RF-09</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>CU-06.3a</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1203,6 +1253,11 @@
           <t>CP-RF-10</t>
         </is>
       </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>CU-06.1e</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1270,6 +1325,11 @@
           <t>CP-RF-11</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>CU-07.1a</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1337,6 +1397,11 @@
           <t>CP-RF-12</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>CU-07.3e</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1404,6 +1469,11 @@
           <t>CP-RF-13</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>CU-03.3a, CU-03.3e</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1471,6 +1541,11 @@
           <t>CP-RF-14</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>CU-03.3b</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1538,6 +1613,11 @@
           <t>CP-RF-15</t>
         </is>
       </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>CU-03.5a</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1605,6 +1685,11 @@
           <t>CP-RF-16</t>
         </is>
       </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>CU-01.2a</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1672,6 +1757,11 @@
           <t>CP-RF-17</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1739,6 +1829,11 @@
           <t>CP-RF-18</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>CU-11.3e</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1806,6 +1901,11 @@
           <t>CP-RF-19</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>CU-08.2e</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1873,6 +1973,11 @@
           <t>CP-RF-20</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>CU-09.2e, CU-09.4e</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1940,6 +2045,11 @@
           <t>CP-RF-21</t>
         </is>
       </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>CU-10.2a, CU-10.3a</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2007,6 +2117,11 @@
           <t>CP-RF-22</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>CU-09.3e</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2074,6 +2189,11 @@
           <t>CP-RF-23</t>
         </is>
       </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>CU-09.4a, CU-09.4f</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2141,6 +2261,11 @@
           <t>CP-RF-24</t>
         </is>
       </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>CU-11.2a, CU-11.2e</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2208,6 +2333,11 @@
           <t>CP-RF-25</t>
         </is>
       </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2275,6 +2405,11 @@
           <t>CP-RF-26</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>CU-04.2a</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2342,6 +2477,11 @@
           <t>CP-RF-27</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2409,6 +2549,11 @@
           <t>CP-RF-28</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2476,6 +2621,11 @@
           <t>CP-RF-29</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>CU-01.5e</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2543,6 +2693,11 @@
           <t>CP-RF-30</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>CU-05.3a</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2610,6 +2765,11 @@
           <t>CP-RF-31</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>CU-06.1a, CU-06.1f</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2677,6 +2837,11 @@
           <t>N/A (Won't have)</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2744,6 +2909,11 @@
           <t>CP-RF-33</t>
         </is>
       </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>CU-06.3e</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2811,6 +2981,11 @@
           <t>CP-RF-34</t>
         </is>
       </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2878,6 +3053,11 @@
           <t>CP-RF-35</t>
         </is>
       </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>CU-01.4a</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2945,6 +3125,11 @@
           <t>CP-RF-36</t>
         </is>
       </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>CU-13.2e</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3012,6 +3197,11 @@
           <t>CP-RF-37</t>
         </is>
       </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>CU-12.2a, CU-14.4e</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3079,6 +3269,11 @@
           <t>CP-RF-38</t>
         </is>
       </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>CU-13.1a, CU-14.4a</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3146,6 +3341,11 @@
           <t>CP-RF-39</t>
         </is>
       </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>CU-13.2e</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3213,6 +3413,11 @@
           <t>CP-RNF-01</t>
         </is>
       </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3280,6 +3485,11 @@
           <t>CP-RNF-02</t>
         </is>
       </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3347,6 +3557,11 @@
           <t>CP-RNF-03</t>
         </is>
       </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3414,6 +3629,11 @@
           <t>CP-RNF-04</t>
         </is>
       </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>CU-02.3a, CU-03.4a</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3481,6 +3701,11 @@
           <t>CP-RNF-05</t>
         </is>
       </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3548,6 +3773,11 @@
           <t>CP-RNF-06</t>
         </is>
       </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3615,6 +3845,11 @@
           <t>CP-RNF-07</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3682,6 +3917,11 @@
           <t>CP-RNF-08</t>
         </is>
       </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3749,6 +3989,11 @@
           <t>CP-RNF-09</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3816,6 +4061,11 @@
           <t>CP-RNF-10</t>
         </is>
       </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3883,6 +4133,11 @@
           <t>CP-RNF-11</t>
         </is>
       </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3950,6 +4205,11 @@
           <t>CP-RNF-12</t>
         </is>
       </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4017,6 +4277,11 @@
           <t>CP-RNF-13</t>
         </is>
       </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4084,6 +4349,11 @@
           <t>CP-RNF-14</t>
         </is>
       </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4151,6 +4421,11 @@
           <t>CP-RNF-15</t>
         </is>
       </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>CU-05.4a, CU-07.3a</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4218,6 +4493,11 @@
           <t>CP-RF-03</t>
         </is>
       </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4285,6 +4565,11 @@
           <t>CP-RF-01</t>
         </is>
       </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4352,6 +4637,11 @@
           <t>CP-RF-04</t>
         </is>
       </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4419,6 +4709,11 @@
           <t>CP-RF-07</t>
         </is>
       </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4486,6 +4781,11 @@
           <t>CP-RF-11</t>
         </is>
       </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4553,6 +4853,11 @@
           <t>CP-RF-29</t>
         </is>
       </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4620,6 +4925,11 @@
           <t>CP-RNF-16</t>
         </is>
       </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4687,6 +4997,11 @@
           <t>CP-RNF-17</t>
         </is>
       </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4754,6 +5069,11 @@
           <t>CP-RNF-18</t>
         </is>
       </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4821,6 +5141,11 @@
           <t>CP-RNF-19</t>
         </is>
       </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4888,6 +5213,11 @@
           <t>CP-RNF-20</t>
         </is>
       </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4953,6 +5283,11 @@
       <c r="M67" t="inlineStr">
         <is>
           <t>CP-RNF-21</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>